<commit_message>
feat(reporter): add custom HTML reporter and integrate test suite configurations
</commit_message>
<xml_diff>
--- a/swarajya-login/swarajya-automation/test_data/login_test_cases.xlsx
+++ b/swarajya-login/swarajya-automation/test_data/login_test_cases.xlsx
@@ -651,6 +651,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:30</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:106: in test_valid_login_and_2fa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'Admin' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="62" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -776,6 +799,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:31</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:106: in test_valid_login_and_2fa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'HR' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -887,7 +933,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-09-03 16:57:30</t>
+          <t>2026-09-08 14:40:18</t>
         </is>
       </c>
     </row>
@@ -946,7 +992,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-08-13 19:55:54</t>
+          <t>2026-09-08 14:40:20</t>
         </is>
       </c>
     </row>
@@ -1000,6 +1046,31 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:53</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:201: in test_general_login_cases
+    login, tfa, _ = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="62" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -1049,19 +1120,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-08-12 16:11:56</t>
+          <t>2026-09-08 14:38:54</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Verified via Manager role</t>
+          <t>tests\test_hr_admin.py:206: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -1119,20 +1200,22 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-13 19:56:22</t>
+          <t>2026-09-08 14:40:39</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>tests\test_login.py:101: in test_2fa_back_to_login_TC_LOGIN_005
-    lp.login(creds["employee_id"], creds["password"])
-pages\login_page.py:66: in login
-    self.enter_employee_id(emp_id)
-pages\login_page.py:54: in enter_employee_id
-    self.employee_id_input.fill(str(emp_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator</t>
+          <t>tests\test_hr_admin.py:212: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -1191,18 +1274,22 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-08-13 19:56:41</t>
+          <t>2026-09-08 14:40:49</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>self = &lt;tests.test_login.TestLoginFlows object at 0x0000020CFB427610&gt;
-page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
-base_url = 'https://swarajya-stg.corecotechnologies.com'
-employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
-    def test_logout_TC_LOGIN_006(self, page, base_url, employee_credentials):
-        """After full login, logging out should land back on the sign-in page."""
-        creds = employee_cre</t>
+          <t>tests\test_hr_admin.py:219: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -1260,15 +1347,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-08-13 19:55:58</t>
+          <t>2026-09-08 14:40:22</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>tests\test_login.py:100: in test_forgot_password_link_TC_LOGIN_007
-    assert "/forgot" in current_url, (
-E   AssertionError: Expected URL to contain '/forgot', got: https://swarajya-stg.corecotechnologies.com/
-E   assert '/forgot' in 'https://swarajya-stg.corecotechnologies.com/'</t>
+          <t>tests\test_hr_admin.py:230: in test_general_login_cases
+    assert "/forgot" in page.url.lower()
+E   AssertionError: assert '/forgot' in 'https://swarajya-stg.corecotechnologies.com/'
+E    +  where 'https://swarajya-stg.corecotechnologies.com/' = &lt;built-in method lower of str object at 0x000001978107D770&gt;()
+E    +    where &lt;built-in method lower of str object at 0x000001978107D770&gt; = 'https://swarajya-stg.corecotechnologies.com/'.lower
+E    +      where 'https://swarajya-stg.corecotechnologies.c</t>
         </is>
       </c>
     </row>
@@ -1318,6 +1407,21 @@
       <c r="J13" s="3" t="inlineStr">
         <is>
           <t>UI</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:58</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Skipped: Alternate-browser validation is not available in the local runner</t>
         </is>
       </c>
     </row>
@@ -1464,6 +1568,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:36</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:137: in test_invalid_employee_id
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'Admin' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="62" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -1515,6 +1642,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:40</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:162: in test_wrong_password
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'Admin' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="62" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1688,6 +1838,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:38</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:137: in test_invalid_employee_id
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'HR' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="62" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1739,6 +1912,29 @@
           <t>UI</t>
         </is>
       </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-08 14:38:42</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>tests\test_hr_admin.py:162: in test_wrong_password
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in credentials.xlsx")
+E   ValueError: Role 'HR' not found in credentials.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="62" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1919,7 +2115,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:01</t>
+          <t>2026-09-08 14:41:01</t>
         </is>
       </c>
     </row>
@@ -1980,7 +2176,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:06</t>
+          <t>2026-09-08 14:41:03</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2237,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:11</t>
+          <t>2026-09-08 14:41:06</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2298,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:15</t>
+          <t>2026-09-08 14:41:08</t>
         </is>
       </c>
     </row>
@@ -2163,12 +2359,19 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:21</t>
+          <t>2026-09-08 14:41:10</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>App trimmed spaces and proceeded to 2FA</t>
+          <t>tests\test_hr_admin.py:268: in test_general_login_cases
+    assert login.get_error_message(timeout=5_000) or "/tfa-authcode/" not in page.url
+E   AssertionError: assert ('' or '/tfa-authcode/' not in 'https://swa...VzVKRQ%3D%3D'
+E    +  where '' = get_error_message(timeout=5000)
+E    +    where get_error_message = &lt;pages.login_page.LoginPage object at 0x00000197FFE22E40&gt;.get_error_message
+E     
+E     '/tfa-authcode/' is contained here:
+E       https://swarajya-stg.corecotechnologies.com/tfa-aut</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2432,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:27</t>
+          <t>2026-09-08 14:41:13</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2302,7 +2505,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:33</t>
+          <t>2026-09-08 14:41:15</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2566,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-08-13 19:57:37</t>
+          <t>2026-09-08 14:41:18</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2422,14 +2625,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K18" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-08-13 19:51:44</t>
+          <t>2026-09-08 14:42:06</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2497,14 +2700,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-08-13 19:51:57</t>
+          <t>2026-09-08 14:42:08</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2572,14 +2775,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-08-13 19:52:09</t>
+          <t>2026-09-08 14:42:10</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2651,7 +2854,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:02</t>
+          <t>2026-09-08 14:42:52</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2710,14 +2913,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-08-13 19:52:21</t>
+          <t>2026-09-08 14:42:14</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2780,25 +2983,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-08-13 19:52:29</t>
+          <t>2026-09-08 14:42:17</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>self = &lt;tests.test_login.TestNegative2FA object at 0x0000020CFB427D90&gt;
-page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/default'&gt;
-base_url = 'https://swarajya-stg.corecotechnologies.com'
-employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
-    def test_wrong_2fa_code_TC_LOGIN_022(self, page, base_url, employee_credentials):
-        """Incorrect 2FA code should not proceed to dashboard."""
-        tfa = self._login_an</t>
+          <t>tests\test_hr_admin.py:328: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -2857,20 +3064,22 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-08-13 19:52:36</t>
+          <t>2026-09-08 14:42:19</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests\test_login.py:676: in test_blank_2fa_code_TC_LOGIN_023
-    login_pg.navigate()
-pages\login_page.py:64: in navigate
-    self.page.goto(url, wait_until="networkidle", timeout=30_000)
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:9875: in goto
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_page.py:560: in goto
-    return await self._main_frame.goto(**locals_to_params(locals()))
-       </t>
+          <t>tests\test_hr_admin.py:334: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -2923,19 +3132,19 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:05</t>
+          <t>2026-09-08 14:42:53</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Skipped: BLOCKED: Cannot reliably control TOTP expiry in automation</t>
+          <t>Skipped: Staging backend accepts any 6-digit numeric OTP (dummy 2FA validator)</t>
         </is>
       </c>
     </row>
@@ -2989,19 +3198,19 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K26" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:09</t>
+          <t>2026-09-08 14:42:53</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Skipped: BLOCKED: Cannot control TOTP rotation timing in automation</t>
+          <t>Skipped: Staging backend accepts any 6-digit numeric OTP (dummy 2FA validator)</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3269,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-08-13 19:52:53</t>
+          <t>2026-09-08 14:42:26</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3124,28 +3333,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-08-13 19:51:54</t>
+          <t>2026-09-08 14:42:28</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>tests\test_login.py:362: in test_repeated_wrong_2fa_TC_LOGIN_027
-    tfa = self._login_and_reach_2fa(page, base_url, employee_credentials)
-          ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-tests\test_login.py:323: in _login_and_reach_2fa
-    lp.login(creds["employee_id"], creds["password"])
-pages\login_page.py:66: in login
-    self.enter_employee_id(emp_id)
-pages\login_page.py:54: in enter_employee_id
-    self.employee_id_input.fill(str(emp_id))
-..\..\..\AppData\Local\Pro</t>
+          <t>tests\test_hr_admin.py:359: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3415,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-08-13 19:53:15</t>
+          <t>2026-09-08 14:42:31</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3276,7 +3486,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-08-13 19:53:19</t>
+          <t>2026-09-08 14:42:33</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3340,19 +3550,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:09</t>
+          <t>2026-09-08 14:39:47</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Skipped: RBAC not implemented in staging</t>
+          <t>tests\test_hr_admin.py:380: in test_general_login_cases
+    login, _, _ = _login_to_tfa(page, base_url, role=role_map[tc_id])
+                  ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not fou</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3631,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:09</t>
+          <t>2026-09-08 14:42:53</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3475,7 +3695,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:09</t>
+          <t>2026-09-08 14:42:53</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3539,7 +3759,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-08-13 19:53:40</t>
+          <t>2026-09-08 14:42:39</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3611,12 +3831,22 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-08-13 19:54:15</t>
+          <t>2026-09-08 14:42:57</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Skipped: BLOCKED: Cannot control server-side session timeout in UI automation</t>
+          <t>tests\test_hr_admin.py:394: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>
@@ -3669,25 +3899,29 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K36" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-08-13 19:53:59</t>
+          <t>2026-09-08 14:42:50</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">self = &lt;tests.test_login.TestSecurityAndSession object at 0x0000020CFB4DD480&gt;
-page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
-base_url = 'https://swarajya-stg.corecotechnologies.com'
-employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
-    def test_back_button_after_logout_TC_LOGIN_035(self, page, base_url, employee_credentials):
-        """Browser back after logout should not expose cached dashboard."""
-        </t>
+          <t>tests\test_hr_admin.py:403: in test_general_login_cases
+    _, tfa, creds = _login_to_tfa(page, base_url, role="Admin")
+                    ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:87: in _login_to_tfa
+    creds = credentials(role)
+            ^^^^^^^^^^^^^^^^^
+tests\test_hr_admin.py:83: in credentials
+    return read_credentials(role)
+           ^^^^^^^^^^^^^^^^^^^^^^
+utils\excel_reader.py:71: in read_credentials
+    raise ValueError(f"Role '{role}' not found in creden</t>
         </is>
       </c>
     </row>

</xml_diff>